<commit_message>
Updates to AC board and pm22V prior to order
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/AC_Board/AC_Board_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/AC_Board/AC_Board_BOM_digikey.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1757255</t>
+          <t>1729131</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -469,22 +469,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>J1,J2,J3</t>
+          <t>AC_Board J1,J2,J3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MSTBA 2,5/3-G-5,08</t>
+          <t>MKDS 1,5/3-5,08</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Phoenix_MSTBA_3</t>
+          <t>TerminalBlock_MKDS_3_P5.08mm</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Term block header 3pos 5.08mm horiz</t>
+          <t>Single-piece PCB screw terminal 3pos 5.08mm side-entry</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PEM01</t>
+          <t>AC_Board PEM01</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PEM01 fuse</t>
+          <t>AC_Board PEM01 fuse</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>AC_Board R1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>AC_Board T1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>AC_Board T2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TH1</t>
+          <t>AC_Board TH1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>